<commit_message>
Update data sources and figures for extended Healthmap period
Replaced Healthmap data files with a new consolidated file covering 2023-05-01 to 2025-10-16. Updated R and Python scripts to use the new data file, adjusted figure scripts (fig1.R, fig2.R, fig3.R, fig4.R) for new data structure, improved plotting logic, and enhanced figure layouts. Removed obsolete data files and added new ignore rules for generated and intermediate files.
</commit_message>
<xml_diff>
--- a/Data/Pertussis case year age.xlsx
+++ b/Data/Pertussis case year age.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://6kmwxn-my.sharepoint.com/personal/kanggle_lkg1116_onmicrosoft_com/Documents/XMU/likangguo/2024/06 pertussis/PertussisIncidence/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://6kmwxn-my.sharepoint.com/personal/kanggle_globalinfectiousdisease_com/Documents/XMU/likangguo/2024/06 pertussis/PertussisIncidence/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="924" documentId="13_ncr:1_{C46EE4FA-0A9A-4805-AEAC-250B1BF7A9E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{665AD5CD-C81E-4842-8FAD-5FC053E7AD47}"/>
+  <xr:revisionPtr revIDLastSave="982" documentId="13_ncr:1_{C46EE4FA-0A9A-4805-AEAC-250B1BF7A9E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C8C413F4-D484-496E-8028-0791FF11CE65}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9850" yWindow="21490" windowWidth="19420" windowHeight="12420" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AU" sheetId="1" r:id="rId1"/>
@@ -382,7 +382,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="0_);[Red]\(0\)"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <name val="等线"/>
@@ -463,7 +463,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -511,6 +511,9 @@
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="差" xfId="1" builtinId="27"/>
@@ -530,14 +533,10 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 主题​​">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 主题">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -575,7 +574,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -681,7 +680,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -823,7 +822,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -831,13 +830,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T10"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:T11"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="24.875" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:20">
       <c r="A1" s="10" t="s">
         <v>88</v>
       </c>
@@ -899,561 +898,623 @@
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A2" s="2">
+    <row r="2" spans="1:20">
+      <c r="A2" s="10">
+        <v>2024</v>
+      </c>
+      <c r="B2" s="21">
+        <v>4729</v>
+      </c>
+      <c r="C2" s="21">
+        <v>12639</v>
+      </c>
+      <c r="D2" s="21">
+        <v>20279</v>
+      </c>
+      <c r="E2" s="21">
+        <v>5006</v>
+      </c>
+      <c r="F2" s="21">
+        <v>2038</v>
+      </c>
+      <c r="G2" s="21">
+        <v>1084</v>
+      </c>
+      <c r="H2" s="21">
+        <v>1023</v>
+      </c>
+      <c r="I2" s="21">
+        <v>1313</v>
+      </c>
+      <c r="J2" s="21">
+        <v>1658</v>
+      </c>
+      <c r="K2" s="21">
+        <v>1789</v>
+      </c>
+      <c r="L2" s="21">
+        <v>1460</v>
+      </c>
+      <c r="M2" s="19">
+        <v>972</v>
+      </c>
+      <c r="N2" s="19">
+        <v>859</v>
+      </c>
+      <c r="O2" s="19">
+        <v>756</v>
+      </c>
+      <c r="P2" s="19">
+        <v>629</v>
+      </c>
+      <c r="Q2" s="19">
+        <v>508</v>
+      </c>
+      <c r="R2" s="19">
+        <v>256</v>
+      </c>
+      <c r="S2" s="19">
+        <v>234</v>
+      </c>
+      <c r="T2" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20">
+      <c r="A3" s="2">
         <v>2023</v>
       </c>
-      <c r="B2">
-        <v>239</v>
-      </c>
-      <c r="C2">
+      <c r="B3" s="19">
+        <v>243</v>
+      </c>
+      <c r="C3" s="19">
         <v>365</v>
       </c>
-      <c r="D2">
-        <v>733</v>
-      </c>
-      <c r="E2">
-        <v>240</v>
-      </c>
-      <c r="F2">
-        <v>100</v>
-      </c>
-      <c r="G2">
+      <c r="D3" s="19">
+        <v>736</v>
+      </c>
+      <c r="E3" s="19">
+        <v>241</v>
+      </c>
+      <c r="F3" s="19">
+        <v>98</v>
+      </c>
+      <c r="G3" s="19">
         <v>58</v>
       </c>
-      <c r="H2">
-        <v>67</v>
-      </c>
-      <c r="I2">
-        <v>73</v>
-      </c>
-      <c r="J2">
+      <c r="H3" s="19">
+        <v>68</v>
+      </c>
+      <c r="I3" s="19">
+        <v>75</v>
+      </c>
+      <c r="J3" s="19">
         <v>85</v>
       </c>
-      <c r="K2">
-        <v>90</v>
-      </c>
-      <c r="L2">
+      <c r="K3" s="19">
+        <v>91</v>
+      </c>
+      <c r="L3" s="19">
         <v>109</v>
       </c>
-      <c r="M2">
+      <c r="M3" s="19">
         <v>58</v>
       </c>
-      <c r="N2">
+      <c r="N3" s="19">
         <v>57</v>
       </c>
-      <c r="O2">
+      <c r="O3" s="19">
         <v>50</v>
       </c>
-      <c r="P2">
+      <c r="P3" s="19">
+        <v>39</v>
+      </c>
+      <c r="Q3" s="19">
+        <v>50</v>
+      </c>
+      <c r="R3" s="19">
+        <v>17</v>
+      </c>
+      <c r="S3" s="19">
+        <v>14</v>
+      </c>
+      <c r="T3" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20">
+      <c r="A4" s="2">
+        <v>2022</v>
+      </c>
+      <c r="B4" s="19">
+        <v>45</v>
+      </c>
+      <c r="C4" s="19">
+        <v>21</v>
+      </c>
+      <c r="D4" s="19">
+        <v>30</v>
+      </c>
+      <c r="E4" s="19">
+        <v>19</v>
+      </c>
+      <c r="F4" s="19">
+        <v>29</v>
+      </c>
+      <c r="G4" s="19">
+        <v>27</v>
+      </c>
+      <c r="H4" s="19">
+        <v>23</v>
+      </c>
+      <c r="I4" s="19">
+        <v>34</v>
+      </c>
+      <c r="J4" s="19">
+        <v>36</v>
+      </c>
+      <c r="K4" s="19">
+        <v>32</v>
+      </c>
+      <c r="L4" s="19">
+        <v>31</v>
+      </c>
+      <c r="M4" s="19">
+        <v>26</v>
+      </c>
+      <c r="N4" s="19">
+        <v>25</v>
+      </c>
+      <c r="O4" s="19">
+        <v>28</v>
+      </c>
+      <c r="P4" s="19">
+        <v>32</v>
+      </c>
+      <c r="Q4" s="19">
+        <v>17</v>
+      </c>
+      <c r="R4" s="19">
+        <v>16</v>
+      </c>
+      <c r="S4" s="19">
+        <v>13</v>
+      </c>
+      <c r="T4" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20">
+      <c r="A5" s="2">
+        <v>2021</v>
+      </c>
+      <c r="B5" s="19">
+        <v>45</v>
+      </c>
+      <c r="C5" s="19">
+        <v>22</v>
+      </c>
+      <c r="D5" s="19">
+        <v>34</v>
+      </c>
+      <c r="E5" s="19">
+        <v>20</v>
+      </c>
+      <c r="F5" s="19">
+        <v>34</v>
+      </c>
+      <c r="G5" s="19">
+        <v>36</v>
+      </c>
+      <c r="H5" s="19">
+        <v>50</v>
+      </c>
+      <c r="I5" s="19">
+        <v>46</v>
+      </c>
+      <c r="J5" s="19">
+        <v>40</v>
+      </c>
+      <c r="K5" s="19">
+        <v>23</v>
+      </c>
+      <c r="L5" s="19">
+        <v>44</v>
+      </c>
+      <c r="M5" s="19">
+        <v>33</v>
+      </c>
+      <c r="N5" s="19">
+        <v>30</v>
+      </c>
+      <c r="O5" s="19">
+        <v>36</v>
+      </c>
+      <c r="P5" s="19">
+        <v>23</v>
+      </c>
+      <c r="Q5" s="19">
+        <v>20</v>
+      </c>
+      <c r="R5" s="19">
+        <v>8</v>
+      </c>
+      <c r="S5" s="19">
+        <v>6</v>
+      </c>
+      <c r="T5" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20">
+      <c r="A6" s="2">
+        <v>2020</v>
+      </c>
+      <c r="B6" s="19">
+        <v>378</v>
+      </c>
+      <c r="C6" s="19">
+        <v>512</v>
+      </c>
+      <c r="D6" s="19">
+        <v>485</v>
+      </c>
+      <c r="E6" s="19">
+        <v>236</v>
+      </c>
+      <c r="F6" s="19">
+        <v>178</v>
+      </c>
+      <c r="G6" s="19">
+        <v>147</v>
+      </c>
+      <c r="H6" s="19">
+        <v>176</v>
+      </c>
+      <c r="I6" s="19">
+        <v>169</v>
+      </c>
+      <c r="J6" s="19">
+        <v>189</v>
+      </c>
+      <c r="K6" s="19">
+        <v>237</v>
+      </c>
+      <c r="L6" s="19">
+        <v>172</v>
+      </c>
+      <c r="M6" s="19">
+        <v>146</v>
+      </c>
+      <c r="N6" s="19">
+        <v>118</v>
+      </c>
+      <c r="O6" s="19">
+        <v>94</v>
+      </c>
+      <c r="P6" s="19">
+        <v>77</v>
+      </c>
+      <c r="Q6" s="19">
+        <v>72</v>
+      </c>
+      <c r="R6" s="19">
         <v>37</v>
       </c>
-      <c r="Q2">
-        <v>50</v>
-      </c>
-      <c r="R2">
-        <v>17</v>
-      </c>
-      <c r="S2">
-        <v>13</v>
-      </c>
-      <c r="T2">
+      <c r="S6" s="19">
+        <v>36</v>
+      </c>
+      <c r="T6" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20">
+      <c r="A7" s="2">
+        <v>2019</v>
+      </c>
+      <c r="B7" s="21">
+        <v>1342</v>
+      </c>
+      <c r="C7" s="21">
+        <v>2625</v>
+      </c>
+      <c r="D7" s="21">
+        <v>2349</v>
+      </c>
+      <c r="E7" s="19">
+        <v>778</v>
+      </c>
+      <c r="F7" s="19">
+        <v>424</v>
+      </c>
+      <c r="G7" s="19">
+        <v>380</v>
+      </c>
+      <c r="H7" s="19">
+        <v>465</v>
+      </c>
+      <c r="I7" s="19">
+        <v>482</v>
+      </c>
+      <c r="J7" s="19">
+        <v>528</v>
+      </c>
+      <c r="K7" s="19">
+        <v>569</v>
+      </c>
+      <c r="L7" s="19">
+        <v>482</v>
+      </c>
+      <c r="M7" s="19">
+        <v>386</v>
+      </c>
+      <c r="N7" s="19">
+        <v>331</v>
+      </c>
+      <c r="O7" s="19">
+        <v>284</v>
+      </c>
+      <c r="P7" s="19">
+        <v>248</v>
+      </c>
+      <c r="Q7" s="19">
+        <v>190</v>
+      </c>
+      <c r="R7" s="19">
+        <v>96</v>
+      </c>
+      <c r="S7" s="19">
+        <v>65</v>
+      </c>
+      <c r="T7" s="19">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A3" s="2">
-        <v>2022</v>
-      </c>
-      <c r="B3">
-        <v>45</v>
-      </c>
-      <c r="C3">
-        <v>22</v>
-      </c>
-      <c r="D3">
-        <v>31</v>
-      </c>
-      <c r="E3">
-        <v>19</v>
-      </c>
-      <c r="F3">
-        <v>28</v>
-      </c>
-      <c r="G3">
-        <v>27</v>
-      </c>
-      <c r="H3">
-        <v>23</v>
-      </c>
-      <c r="I3">
-        <v>34</v>
-      </c>
-      <c r="J3">
-        <v>35</v>
-      </c>
-      <c r="K3">
-        <v>32</v>
-      </c>
-      <c r="L3">
-        <v>30</v>
-      </c>
-      <c r="M3">
-        <v>26</v>
-      </c>
-      <c r="N3">
-        <v>25</v>
-      </c>
-      <c r="O3">
-        <v>28</v>
-      </c>
-      <c r="P3">
-        <v>32</v>
-      </c>
-      <c r="Q3">
-        <v>17</v>
-      </c>
-      <c r="R3">
-        <v>16</v>
-      </c>
-      <c r="S3">
-        <v>13</v>
-      </c>
-      <c r="T3">
+    <row r="8" spans="1:20">
+      <c r="A8" s="2">
+        <v>2018</v>
+      </c>
+      <c r="B8" s="21">
+        <v>1514</v>
+      </c>
+      <c r="C8" s="21">
+        <v>3080</v>
+      </c>
+      <c r="D8" s="21">
+        <v>2193</v>
+      </c>
+      <c r="E8" s="19">
+        <v>663</v>
+      </c>
+      <c r="F8" s="19">
+        <v>386</v>
+      </c>
+      <c r="G8" s="19">
+        <v>409</v>
+      </c>
+      <c r="H8" s="19">
+        <v>426</v>
+      </c>
+      <c r="I8" s="19">
+        <v>518</v>
+      </c>
+      <c r="J8" s="19">
+        <v>592</v>
+      </c>
+      <c r="K8" s="19">
+        <v>581</v>
+      </c>
+      <c r="L8" s="19">
+        <v>492</v>
+      </c>
+      <c r="M8" s="19">
+        <v>431</v>
+      </c>
+      <c r="N8" s="19">
+        <v>378</v>
+      </c>
+      <c r="O8" s="19">
+        <v>317</v>
+      </c>
+      <c r="P8" s="19">
+        <v>273</v>
+      </c>
+      <c r="Q8" s="19">
+        <v>166</v>
+      </c>
+      <c r="R8" s="19">
+        <v>85</v>
+      </c>
+      <c r="S8" s="19">
+        <v>77</v>
+      </c>
+      <c r="T8" s="19">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A4" s="2">
-        <v>2021</v>
-      </c>
-      <c r="B4">
-        <v>45</v>
-      </c>
-      <c r="C4">
-        <v>22</v>
-      </c>
-      <c r="D4">
-        <v>34</v>
-      </c>
-      <c r="E4">
-        <v>20</v>
-      </c>
-      <c r="F4">
-        <v>34</v>
-      </c>
-      <c r="G4">
-        <v>36</v>
-      </c>
-      <c r="H4">
-        <v>50</v>
-      </c>
-      <c r="I4">
-        <v>46</v>
-      </c>
-      <c r="J4">
-        <v>40</v>
-      </c>
-      <c r="K4">
-        <v>23</v>
-      </c>
-      <c r="L4">
-        <v>44</v>
-      </c>
-      <c r="M4">
-        <v>33</v>
-      </c>
-      <c r="N4">
-        <v>30</v>
-      </c>
-      <c r="O4">
-        <v>36</v>
-      </c>
-      <c r="P4">
-        <v>23</v>
-      </c>
-      <c r="Q4">
-        <v>20</v>
-      </c>
-      <c r="R4">
-        <v>8</v>
-      </c>
-      <c r="S4">
-        <v>6</v>
-      </c>
-      <c r="T4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A5" s="2">
-        <v>2020</v>
-      </c>
-      <c r="B5">
+    <row r="9" spans="1:20">
+      <c r="A9" s="2">
+        <v>2017</v>
+      </c>
+      <c r="B9" s="21">
+        <v>1747</v>
+      </c>
+      <c r="C9" s="21">
+        <v>2275</v>
+      </c>
+      <c r="D9" s="21">
+        <v>1740</v>
+      </c>
+      <c r="E9" s="19">
+        <v>738</v>
+      </c>
+      <c r="F9" s="19">
         <v>377</v>
       </c>
-      <c r="C5">
-        <v>512</v>
-      </c>
-      <c r="D5">
-        <v>485</v>
-      </c>
-      <c r="E5">
-        <v>236</v>
-      </c>
-      <c r="F5">
-        <v>178</v>
-      </c>
-      <c r="G5">
-        <v>147</v>
-      </c>
-      <c r="H5">
-        <v>175</v>
-      </c>
-      <c r="I5">
-        <v>169</v>
-      </c>
-      <c r="J5">
-        <v>189</v>
-      </c>
-      <c r="K5">
-        <v>237</v>
-      </c>
-      <c r="L5">
-        <v>172</v>
-      </c>
-      <c r="M5">
-        <v>146</v>
-      </c>
-      <c r="N5">
-        <v>118</v>
-      </c>
-      <c r="O5">
-        <v>94</v>
-      </c>
-      <c r="P5">
-        <v>77</v>
-      </c>
-      <c r="Q5">
-        <v>72</v>
-      </c>
-      <c r="R5">
-        <v>37</v>
-      </c>
-      <c r="S5">
-        <v>36</v>
-      </c>
-      <c r="T5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A6" s="2">
-        <v>2019</v>
-      </c>
-      <c r="B6" s="3">
-        <v>1342</v>
-      </c>
-      <c r="C6" s="3">
-        <v>2624</v>
-      </c>
-      <c r="D6" s="3">
-        <v>2350</v>
-      </c>
-      <c r="E6">
-        <v>778</v>
-      </c>
-      <c r="F6">
-        <v>424</v>
-      </c>
-      <c r="G6">
-        <v>380</v>
-      </c>
-      <c r="H6">
-        <v>465</v>
-      </c>
-      <c r="I6">
-        <v>482</v>
-      </c>
-      <c r="J6">
+      <c r="G9" s="19">
+        <v>457</v>
+      </c>
+      <c r="H9" s="19">
         <v>528</v>
       </c>
-      <c r="K6">
-        <v>569</v>
-      </c>
-      <c r="L6">
-        <v>482</v>
-      </c>
-      <c r="M6">
+      <c r="I9" s="19">
+        <v>541</v>
+      </c>
+      <c r="J9" s="19">
+        <v>636</v>
+      </c>
+      <c r="K9" s="19">
+        <v>623</v>
+      </c>
+      <c r="L9" s="19">
+        <v>500</v>
+      </c>
+      <c r="M9" s="19">
+        <v>472</v>
+      </c>
+      <c r="N9" s="19">
+        <v>408</v>
+      </c>
+      <c r="O9" s="19">
         <v>386</v>
       </c>
-      <c r="N6">
-        <v>331</v>
-      </c>
-      <c r="O6">
-        <v>284</v>
-      </c>
-      <c r="P6">
-        <v>248</v>
-      </c>
-      <c r="Q6">
-        <v>190</v>
-      </c>
-      <c r="R6">
-        <v>96</v>
-      </c>
-      <c r="S6">
-        <v>65</v>
-      </c>
-      <c r="T6">
+      <c r="P9" s="19">
+        <v>340</v>
+      </c>
+      <c r="Q9" s="19">
+        <v>229</v>
+      </c>
+      <c r="R9" s="19">
+        <v>120</v>
+      </c>
+      <c r="S9" s="19">
+        <v>117</v>
+      </c>
+      <c r="T9" s="19">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A7" s="2">
-        <v>2018</v>
-      </c>
-      <c r="B7" s="3">
-        <v>1514</v>
-      </c>
-      <c r="C7" s="3">
-        <v>3080</v>
-      </c>
-      <c r="D7" s="3">
-        <v>2193</v>
-      </c>
-      <c r="E7">
-        <v>663</v>
-      </c>
-      <c r="F7">
-        <v>386</v>
-      </c>
-      <c r="G7">
-        <v>409</v>
-      </c>
-      <c r="H7">
-        <v>426</v>
-      </c>
-      <c r="I7">
-        <v>518</v>
-      </c>
-      <c r="J7">
-        <v>592</v>
-      </c>
-      <c r="K7">
-        <v>581</v>
-      </c>
-      <c r="L7">
-        <v>492</v>
-      </c>
-      <c r="M7">
-        <v>431</v>
-      </c>
-      <c r="N7">
-        <v>378</v>
-      </c>
-      <c r="O7">
-        <v>317</v>
-      </c>
-      <c r="P7">
-        <v>273</v>
-      </c>
-      <c r="Q7">
-        <v>166</v>
-      </c>
-      <c r="R7">
-        <v>85</v>
-      </c>
-      <c r="S7">
-        <v>77</v>
-      </c>
-      <c r="T7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A8" s="2">
-        <v>2017</v>
-      </c>
-      <c r="B8" s="3">
-        <v>1748</v>
-      </c>
-      <c r="C8" s="3">
-        <v>2275</v>
-      </c>
-      <c r="D8" s="3">
-        <v>1740</v>
-      </c>
-      <c r="E8">
-        <v>738</v>
-      </c>
-      <c r="F8">
-        <v>377</v>
-      </c>
-      <c r="G8">
-        <v>457</v>
-      </c>
-      <c r="H8">
+    <row r="10" spans="1:20">
+      <c r="A10" s="2">
+        <v>2016</v>
+      </c>
+      <c r="B10" s="21">
+        <v>2908</v>
+      </c>
+      <c r="C10" s="21">
+        <v>4052</v>
+      </c>
+      <c r="D10" s="21">
+        <v>3535</v>
+      </c>
+      <c r="E10" s="21">
+        <v>1078</v>
+      </c>
+      <c r="F10" s="19">
+        <v>686</v>
+      </c>
+      <c r="G10" s="19">
+        <v>701</v>
+      </c>
+      <c r="H10" s="19">
+        <v>787</v>
+      </c>
+      <c r="I10" s="19">
+        <v>878</v>
+      </c>
+      <c r="J10" s="21">
+        <v>1043</v>
+      </c>
+      <c r="K10" s="19">
+        <v>887</v>
+      </c>
+      <c r="L10" s="19">
+        <v>723</v>
+      </c>
+      <c r="M10" s="19">
+        <v>664</v>
+      </c>
+      <c r="N10" s="19">
+        <v>583</v>
+      </c>
+      <c r="O10" s="19">
+        <v>612</v>
+      </c>
+      <c r="P10" s="19">
+        <v>436</v>
+      </c>
+      <c r="Q10" s="19">
+        <v>277</v>
+      </c>
+      <c r="R10" s="19">
+        <v>127</v>
+      </c>
+      <c r="S10" s="19">
+        <v>138</v>
+      </c>
+      <c r="T10" s="19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20">
+      <c r="A11" s="2">
+        <v>2015</v>
+      </c>
+      <c r="B11" s="21">
+        <v>2894</v>
+      </c>
+      <c r="C11" s="21">
+        <v>4464</v>
+      </c>
+      <c r="D11" s="21">
+        <v>4293</v>
+      </c>
+      <c r="E11" s="21">
+        <v>1108</v>
+      </c>
+      <c r="F11" s="19">
+        <v>633</v>
+      </c>
+      <c r="G11" s="19">
+        <v>656</v>
+      </c>
+      <c r="H11" s="19">
+        <v>769</v>
+      </c>
+      <c r="I11" s="19">
+        <v>920</v>
+      </c>
+      <c r="J11" s="21">
+        <v>1222</v>
+      </c>
+      <c r="K11" s="21">
+        <v>1140</v>
+      </c>
+      <c r="L11" s="19">
+        <v>894</v>
+      </c>
+      <c r="M11" s="19">
+        <v>782</v>
+      </c>
+      <c r="N11" s="19">
+        <v>781</v>
+      </c>
+      <c r="O11" s="19">
+        <v>749</v>
+      </c>
+      <c r="P11" s="19">
         <v>528</v>
       </c>
-      <c r="I8">
-        <v>541</v>
-      </c>
-      <c r="J8">
-        <v>636</v>
-      </c>
-      <c r="K8">
-        <v>623</v>
-      </c>
-      <c r="L8">
-        <v>499</v>
-      </c>
-      <c r="M8">
-        <v>472</v>
-      </c>
-      <c r="N8">
-        <v>408</v>
-      </c>
-      <c r="O8">
-        <v>386</v>
-      </c>
-      <c r="P8">
-        <v>340</v>
-      </c>
-      <c r="Q8">
-        <v>229</v>
-      </c>
-      <c r="R8">
-        <v>120</v>
-      </c>
-      <c r="S8">
-        <v>117</v>
-      </c>
-      <c r="T8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A9" s="2">
-        <v>2016</v>
-      </c>
-      <c r="B9" s="3">
-        <v>2909</v>
-      </c>
-      <c r="C9" s="3">
-        <v>4052</v>
-      </c>
-      <c r="D9" s="3">
-        <v>3535</v>
-      </c>
-      <c r="E9" s="3">
-        <v>1078</v>
-      </c>
-      <c r="F9">
-        <v>686</v>
-      </c>
-      <c r="G9">
-        <v>701</v>
-      </c>
-      <c r="H9">
-        <v>787</v>
-      </c>
-      <c r="I9">
-        <v>878</v>
-      </c>
-      <c r="J9" s="3">
-        <v>1043</v>
-      </c>
-      <c r="K9">
-        <v>887</v>
-      </c>
-      <c r="L9">
-        <v>723</v>
-      </c>
-      <c r="M9">
-        <v>663</v>
-      </c>
-      <c r="N9">
-        <v>583</v>
-      </c>
-      <c r="O9">
-        <v>612</v>
-      </c>
-      <c r="P9">
-        <v>436</v>
-      </c>
-      <c r="Q9">
-        <v>277</v>
-      </c>
-      <c r="R9">
-        <v>127</v>
-      </c>
-      <c r="S9">
-        <v>138</v>
-      </c>
-      <c r="T9">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A10" s="2">
-        <v>2015</v>
-      </c>
-      <c r="B10" s="3">
-        <v>2894</v>
-      </c>
-      <c r="C10" s="3">
-        <v>4464</v>
-      </c>
-      <c r="D10" s="3">
-        <v>4293</v>
-      </c>
-      <c r="E10" s="3">
-        <v>1108</v>
-      </c>
-      <c r="F10">
-        <v>633</v>
-      </c>
-      <c r="G10">
-        <v>656</v>
-      </c>
-      <c r="H10">
-        <v>770</v>
-      </c>
-      <c r="I10">
-        <v>920</v>
-      </c>
-      <c r="J10" s="3">
-        <v>1222</v>
-      </c>
-      <c r="K10" s="3">
-        <v>1140</v>
-      </c>
-      <c r="L10">
-        <v>893</v>
-      </c>
-      <c r="M10">
-        <v>782</v>
-      </c>
-      <c r="N10">
-        <v>781</v>
-      </c>
-      <c r="O10">
-        <v>749</v>
-      </c>
-      <c r="P10">
-        <v>527</v>
-      </c>
-      <c r="Q10">
+      <c r="Q11" s="19">
         <v>367</v>
       </c>
-      <c r="R10">
+      <c r="R11" s="19">
         <v>203</v>
       </c>
-      <c r="S10">
+      <c r="S11" s="19">
         <v>168</v>
       </c>
-      <c r="T10">
+      <c r="T11" s="19">
         <v>0</v>
       </c>
     </row>
@@ -1467,14 +1528,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26E2D9B1-1E5E-45A5-B501-433EB35DEFF4}">
   <dimension ref="A1:AD10"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="4" width="13.375" customWidth="1"/>
-    <col min="5" max="5" width="11.625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.375" bestFit="1" customWidth="1"/>
+    <col min="1" max="4" width="13.33203125" customWidth="1"/>
+    <col min="5" max="5" width="11.58203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="12" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:30" s="12" customFormat="1">
       <c r="A1" s="10" t="s">
         <v>88</v>
       </c>
@@ -1566,7 +1627,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:30">
       <c r="A2" s="1">
         <v>2023</v>
       </c>
@@ -1678,7 +1739,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:30">
       <c r="A3" s="1">
         <v>2022</v>
       </c>
@@ -1723,7 +1784,7 @@
       <c r="AC3" s="5"/>
       <c r="AD3" s="5"/>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:30">
       <c r="A4" s="1">
         <v>2021</v>
       </c>
@@ -1781,7 +1842,7 @@
       <c r="AC4" s="5"/>
       <c r="AD4" s="5"/>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:30">
       <c r="A5" s="2">
         <v>2020</v>
       </c>
@@ -1867,7 +1928,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:30">
       <c r="A6" s="2">
         <v>2019</v>
       </c>
@@ -1953,7 +2014,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:30">
       <c r="A7" s="2">
         <v>2018</v>
       </c>
@@ -2039,7 +2100,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:30">
       <c r="A8" s="2">
         <v>2017</v>
       </c>
@@ -2125,7 +2186,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:30">
       <c r="A9" s="2">
         <v>2016</v>
       </c>
@@ -2211,7 +2272,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:30">
       <c r="A10" s="2">
         <v>2015</v>
       </c>
@@ -2306,13 +2367,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7BC46BA-B415-4BA1-8C07-32B789ED57F5}">
-  <dimension ref="A1:J10"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:J11"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="3" max="3" width="9.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10">
       <c r="A1" s="10" t="s">
         <v>88</v>
       </c>
@@ -2344,7 +2405,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10">
       <c r="A2">
         <v>2015</v>
       </c>
@@ -2373,7 +2434,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10">
       <c r="A3">
         <v>2016</v>
       </c>
@@ -2402,7 +2463,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10">
       <c r="A4">
         <v>2017</v>
       </c>
@@ -2431,7 +2492,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10">
       <c r="A5">
         <v>2018</v>
       </c>
@@ -2460,7 +2521,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10">
       <c r="A6">
         <v>2019</v>
       </c>
@@ -2489,7 +2550,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10">
       <c r="A7">
         <v>2020</v>
       </c>
@@ -2514,7 +2575,7 @@
         <v>2342</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10">
       <c r="A8">
         <v>2021</v>
       </c>
@@ -2539,7 +2600,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10">
       <c r="A9">
         <v>2022</v>
       </c>
@@ -2564,7 +2625,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10">
       <c r="A10">
         <v>2023</v>
       </c>
@@ -2587,6 +2648,27 @@
       <c r="I10" s="18"/>
       <c r="J10" s="18">
         <v>453</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="A11">
+        <v>2024</v>
+      </c>
+      <c r="B11" s="18">
+        <f>433+231+229</f>
+        <v>893</v>
+      </c>
+      <c r="C11" s="18">
+        <v>881</v>
+      </c>
+      <c r="D11" s="18">
+        <v>1657</v>
+      </c>
+      <c r="E11" s="18">
+        <v>2707</v>
+      </c>
+      <c r="J11" s="18">
+        <v>8756</v>
       </c>
     </row>
   </sheetData>
@@ -2598,14 +2680,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1ACAAF4F-F540-404D-8EBE-0EF1E094777F}">
-  <dimension ref="A1:M10"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:M11"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="16.75" customWidth="1"/>
     <col min="12" max="12" width="9.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13">
       <c r="A1" s="10" t="s">
         <v>88</v>
       </c>
@@ -2646,12 +2728,13 @@
         <v>58</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" s="6">
-        <v>2023</v>
-      </c>
-      <c r="B2" s="6">
-        <v>729</v>
+    <row r="2" spans="1:13">
+      <c r="A2" s="10">
+        <v>2024</v>
+      </c>
+      <c r="B2" s="11">
+        <f>1573+1150</f>
+        <v>2723</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
@@ -2659,29 +2742,26 @@
       <c r="F2" s="7"/>
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
-      <c r="I2" s="10">
-        <v>2</v>
-      </c>
-      <c r="J2">
-        <v>1762</v>
-      </c>
-      <c r="K2">
-        <v>636</v>
-      </c>
-      <c r="L2">
-        <v>1014</v>
-      </c>
-      <c r="M2">
-        <v>1468</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="I2" s="10"/>
+      <c r="J2" s="4">
+        <v>6539</v>
+      </c>
+      <c r="K2" s="4">
+        <v>4945</v>
+      </c>
+      <c r="L2" s="4">
+        <v>15194</v>
+      </c>
+      <c r="M2" s="4">
+        <v>6026</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
       <c r="A3" s="6">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B3" s="6">
-        <f>130+139</f>
-        <v>269</v>
+        <v>729</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
@@ -2690,221 +2770,251 @@
       <c r="G3" s="7"/>
       <c r="H3" s="7"/>
       <c r="I3" s="10">
+        <v>2</v>
+      </c>
+      <c r="J3">
+        <v>1762</v>
+      </c>
+      <c r="K3">
+        <v>636</v>
+      </c>
+      <c r="L3">
+        <v>1014</v>
+      </c>
+      <c r="M3">
+        <v>1468</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="6">
+        <v>2022</v>
+      </c>
+      <c r="B4" s="6">
+        <f>130+139</f>
+        <v>269</v>
+      </c>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="10">
         <v>1</v>
       </c>
-      <c r="J3">
+      <c r="J4">
         <v>622</v>
       </c>
-      <c r="K3">
+      <c r="K4">
         <v>176</v>
       </c>
-      <c r="L3">
+      <c r="L4">
         <v>231</v>
       </c>
-      <c r="M3">
+      <c r="M4">
         <v>1089</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A4" s="6">
+    <row r="5" spans="1:13">
+      <c r="A5" s="6">
         <v>2021</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B5" s="6">
         <v>177</v>
       </c>
-      <c r="C4" s="11">
+      <c r="C5" s="11">
         <v>378</v>
       </c>
-      <c r="D4" s="11">
+      <c r="D5" s="11">
         <v>232</v>
       </c>
-      <c r="E4" s="11">
+      <c r="E5" s="11">
         <v>179</v>
       </c>
-      <c r="F4" s="11">
+      <c r="F5" s="11">
         <v>262</v>
       </c>
-      <c r="G4" s="11">
+      <c r="G5" s="11">
         <v>603</v>
       </c>
-      <c r="H4" s="11">
+      <c r="H5" s="11">
         <v>283</v>
       </c>
-      <c r="I4" s="10">
+      <c r="I5" s="10">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" s="6">
+    <row r="6" spans="1:13">
+      <c r="A6" s="6">
         <v>2020</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B6" s="8">
         <v>698</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C6" s="9">
         <v>983</v>
       </c>
-      <c r="D5" s="9">
+      <c r="D6" s="9">
         <v>1828</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E6" s="6">
         <v>1078</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F6" s="6">
         <v>366</v>
       </c>
-      <c r="G5" s="6">
+      <c r="G6" s="6">
         <v>774</v>
       </c>
-      <c r="H5" s="6">
+      <c r="H6" s="6">
         <v>388</v>
       </c>
-      <c r="I5" s="6">
+      <c r="I6" s="6">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A6" s="6">
+    <row r="7" spans="1:13">
+      <c r="A7" s="6">
         <v>2019</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B7" s="9">
         <v>2183</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C7" s="9">
         <v>2876</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D7" s="9">
         <v>5874</v>
       </c>
-      <c r="E6" s="9">
+      <c r="E7" s="9">
         <v>3717</v>
       </c>
-      <c r="F6" s="9">
+      <c r="F7" s="9">
         <v>1053</v>
       </c>
-      <c r="G6" s="9">
+      <c r="G7" s="9">
         <v>2030</v>
       </c>
-      <c r="H6" s="9">
+      <c r="H7" s="9">
         <v>864</v>
       </c>
-      <c r="I6" s="9">
+      <c r="I7" s="9">
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A7" s="6">
+    <row r="8" spans="1:13">
+      <c r="A8" s="6">
         <v>2018</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B8" s="9">
         <v>1995</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C8" s="9">
         <v>2431</v>
       </c>
-      <c r="D7" s="9">
+      <c r="D8" s="9">
         <v>4742</v>
       </c>
-      <c r="E7" s="9">
+      <c r="E8" s="9">
         <v>3212</v>
       </c>
-      <c r="F7" s="9">
+      <c r="F8" s="9">
         <v>925</v>
       </c>
-      <c r="G7" s="9">
+      <c r="G8" s="9">
         <v>1629</v>
       </c>
-      <c r="H7" s="9">
+      <c r="H8" s="9">
         <v>652</v>
       </c>
-      <c r="I7" s="9">
+      <c r="I8" s="9">
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A8" s="6">
+    <row r="9" spans="1:13">
+      <c r="A9" s="6">
         <v>2017</v>
       </c>
-      <c r="B8" s="9">
+      <c r="B9" s="9">
         <v>2237</v>
       </c>
-      <c r="C8" s="9">
+      <c r="C9" s="9">
         <v>2779</v>
       </c>
-      <c r="D8" s="9">
+      <c r="D9" s="9">
         <v>6015</v>
       </c>
-      <c r="E8" s="9">
+      <c r="E9" s="9">
         <v>4204</v>
       </c>
-      <c r="F8" s="9">
+      <c r="F9" s="9">
         <v>1035</v>
       </c>
-      <c r="G8" s="9">
+      <c r="G9" s="9">
         <v>1924</v>
       </c>
-      <c r="H8" s="9">
+      <c r="H9" s="9">
         <v>739</v>
       </c>
-      <c r="I8" s="9">
+      <c r="I9" s="9">
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A9" s="6">
+    <row r="10" spans="1:13">
+      <c r="A10" s="6">
         <v>2016</v>
       </c>
-      <c r="B9" s="9">
+      <c r="B10" s="9">
         <v>2020</v>
       </c>
-      <c r="C9" s="9">
+      <c r="C10" s="9">
         <v>2435</v>
       </c>
-      <c r="D9" s="9">
+      <c r="D10" s="9">
         <v>5833</v>
       </c>
-      <c r="E9" s="9">
+      <c r="E10" s="9">
         <v>3998</v>
       </c>
-      <c r="F9" s="9">
+      <c r="F10" s="9">
         <v>1094</v>
       </c>
-      <c r="G9" s="9">
+      <c r="G10" s="9">
         <v>1905</v>
       </c>
-      <c r="H9" s="9">
+      <c r="H10" s="9">
         <v>657</v>
       </c>
-      <c r="I9" s="9">
+      <c r="I10" s="9">
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A10" s="6">
+    <row r="11" spans="1:13">
+      <c r="A11" s="6">
         <v>2015</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B11" s="9">
         <v>2672</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C11" s="9">
         <v>2806</v>
       </c>
-      <c r="D10" s="9">
+      <c r="D11" s="9">
         <v>6870</v>
       </c>
-      <c r="E10" s="9">
+      <c r="E11" s="9">
         <v>4193</v>
       </c>
-      <c r="F10" s="9">
+      <c r="F11" s="9">
         <v>1293</v>
       </c>
-      <c r="G10" s="9">
+      <c r="G11" s="9">
         <v>2154</v>
       </c>
-      <c r="H10" s="9">
+      <c r="H11" s="9">
         <v>736</v>
       </c>
-      <c r="I10" s="9">
+      <c r="I11" s="9">
         <v>38</v>
       </c>
     </row>
@@ -2917,13 +3027,13 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE4C6641-471C-48E4-AB1A-90459E3398B2}">
-  <dimension ref="A1:L11"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:L12"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="11.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12">
       <c r="A1" s="10" t="s">
         <v>88</v>
       </c>
@@ -2961,348 +3071,386 @@
         <v>65</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A2">
+    <row r="2" spans="1:12">
+      <c r="A2" s="10">
+        <v>2024</v>
+      </c>
+      <c r="B2" s="11">
+        <v>120</v>
+      </c>
+      <c r="C2" s="6">
+        <v>242</v>
+      </c>
+      <c r="D2" s="11">
+        <v>294</v>
+      </c>
+      <c r="E2" s="11">
+        <v>306</v>
+      </c>
+      <c r="F2" s="1">
+        <v>158</v>
+      </c>
+      <c r="G2" s="10">
+        <v>128</v>
+      </c>
+      <c r="H2" s="10">
+        <v>132</v>
+      </c>
+      <c r="I2" s="10">
+        <v>148</v>
+      </c>
+      <c r="J2" s="10">
+        <v>112</v>
+      </c>
+      <c r="K2" s="10">
+        <v>60</v>
+      </c>
+      <c r="L2" s="10">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3">
         <v>2023</v>
       </c>
-      <c r="B2" s="6">
+      <c r="B3" s="6">
         <v>31</v>
       </c>
-      <c r="C2" s="6">
+      <c r="C3" s="6">
         <v>18</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D3" s="6">
         <v>12</v>
       </c>
-      <c r="E2" s="6">
+      <c r="E3" s="6">
         <v>16</v>
       </c>
-      <c r="F2" s="6">
+      <c r="F3" s="6">
         <v>5</v>
       </c>
-      <c r="G2" s="6">
+      <c r="G3" s="6">
         <v>12</v>
       </c>
-      <c r="H2" s="6">
+      <c r="H3" s="6">
         <v>14</v>
       </c>
-      <c r="I2" s="6">
+      <c r="I3" s="6">
         <v>14</v>
       </c>
-      <c r="J2" s="6">
+      <c r="J3" s="6">
         <v>8</v>
       </c>
-      <c r="K2" s="6">
+      <c r="K3" s="6">
         <v>7</v>
-      </c>
-      <c r="L2" s="6">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A3">
-        <v>2022</v>
-      </c>
-      <c r="B3" s="6">
-        <v>1</v>
-      </c>
-      <c r="C3" s="6">
-        <v>1</v>
-      </c>
-      <c r="D3" s="6">
-        <v>1</v>
-      </c>
-      <c r="E3" s="6">
-        <v>2</v>
-      </c>
-      <c r="F3" s="6">
-        <v>2</v>
-      </c>
-      <c r="G3" s="6">
-        <v>1</v>
-      </c>
-      <c r="H3" s="6">
-        <v>3</v>
-      </c>
-      <c r="I3" s="6">
-        <v>0</v>
-      </c>
-      <c r="J3" s="6">
-        <v>2</v>
-      </c>
-      <c r="K3" s="6">
-        <v>1</v>
       </c>
       <c r="L3" s="6">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12">
       <c r="A4">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B4" s="6">
         <v>1</v>
       </c>
       <c r="C4" s="6">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D4" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4" s="6">
         <v>2</v>
       </c>
-      <c r="F4" s="6"/>
+      <c r="F4" s="6">
+        <v>2</v>
+      </c>
       <c r="G4" s="6">
+        <v>1</v>
+      </c>
+      <c r="H4" s="6">
+        <v>3</v>
+      </c>
+      <c r="I4" s="6">
+        <v>0</v>
+      </c>
+      <c r="J4" s="6">
+        <v>2</v>
+      </c>
+      <c r="K4" s="6">
+        <v>1</v>
+      </c>
+      <c r="L4" s="6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5">
+        <v>2021</v>
+      </c>
+      <c r="B5" s="6">
+        <v>1</v>
+      </c>
+      <c r="C5" s="6">
+        <v>7</v>
+      </c>
+      <c r="D5" s="6">
+        <v>2</v>
+      </c>
+      <c r="E5" s="6">
+        <v>2</v>
+      </c>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6">
         <v>5</v>
       </c>
-      <c r="H4" s="6">
+      <c r="H5" s="6">
         <v>5</v>
       </c>
-      <c r="I4" s="6">
+      <c r="I5" s="6">
         <v>6</v>
       </c>
-      <c r="J4" s="6">
+      <c r="J5" s="6">
         <v>6</v>
       </c>
-      <c r="K4" s="6">
+      <c r="K5" s="6">
         <v>2</v>
       </c>
-      <c r="L4" s="6">
+      <c r="L5" s="6">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A5">
+    <row r="6" spans="1:12">
+      <c r="A6">
         <v>2020</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B6" s="6">
         <v>16</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C6" s="6">
         <v>29</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D6" s="6">
         <v>15</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E6" s="6">
         <v>16</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F6" s="6">
         <v>5</v>
       </c>
-      <c r="G5" s="6">
+      <c r="G6" s="6">
         <v>19</v>
       </c>
-      <c r="H5" s="6">
+      <c r="H6" s="6">
         <v>16</v>
       </c>
-      <c r="I5" s="6">
+      <c r="I6" s="6">
         <v>17</v>
       </c>
-      <c r="J5" s="6">
+      <c r="J6" s="6">
         <v>24</v>
       </c>
-      <c r="K5" s="6">
+      <c r="K6" s="6">
         <v>9</v>
       </c>
-      <c r="L5" s="6">
+      <c r="L6" s="6">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A6">
+    <row r="7" spans="1:12">
+      <c r="A7">
         <v>2019</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B7" s="6">
         <v>88</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C7" s="6">
         <v>168</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D7" s="6">
         <v>115</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E7" s="6">
         <v>98</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F7" s="6">
         <v>70</v>
       </c>
-      <c r="G6" s="6">
+      <c r="G7" s="6">
         <v>94</v>
       </c>
-      <c r="H6" s="6">
+      <c r="H7" s="6">
         <v>120</v>
       </c>
-      <c r="I6" s="6">
+      <c r="I7" s="6">
         <v>154</v>
       </c>
-      <c r="J6" s="6">
+      <c r="J7" s="6">
         <v>120</v>
       </c>
-      <c r="K6" s="6">
+      <c r="K7" s="6">
         <v>106</v>
       </c>
-      <c r="L6" s="6">
+      <c r="L7" s="6">
         <v>73</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A7">
+    <row r="8" spans="1:12">
+      <c r="A8">
         <v>2018</v>
       </c>
-      <c r="B7" s="6">
+      <c r="B8" s="6">
         <v>184</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C8" s="6">
         <v>370</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D8" s="6">
         <v>407</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E8" s="6">
         <v>306</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F8" s="6">
         <v>192</v>
       </c>
-      <c r="G7" s="6">
+      <c r="G8" s="6">
         <v>254</v>
       </c>
-      <c r="H7" s="6">
+      <c r="H8" s="6">
         <v>296</v>
       </c>
-      <c r="I7" s="6">
+      <c r="I8" s="6">
         <v>372</v>
       </c>
-      <c r="J7" s="6">
+      <c r="J8" s="6">
         <v>274</v>
       </c>
-      <c r="K7" s="6">
+      <c r="K8" s="6">
         <v>163</v>
       </c>
-      <c r="L7" s="6">
+      <c r="L8" s="6">
         <v>134</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A8">
+    <row r="9" spans="1:12">
+      <c r="A9">
         <v>2017</v>
       </c>
-      <c r="B8" s="6">
+      <c r="B9" s="6">
         <v>129</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C9" s="6">
         <v>222</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D9" s="6">
         <v>295</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E9" s="6">
         <v>269</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F9" s="6">
         <v>202</v>
       </c>
-      <c r="G8" s="6">
+      <c r="G9" s="6">
         <v>151</v>
       </c>
-      <c r="H8" s="6">
+      <c r="H9" s="6">
         <v>199</v>
       </c>
-      <c r="I8" s="6">
+      <c r="I9" s="6">
         <v>269</v>
       </c>
-      <c r="J8" s="6">
+      <c r="J9" s="6">
         <v>198</v>
       </c>
-      <c r="K8" s="6">
+      <c r="K9" s="6">
         <v>120</v>
       </c>
-      <c r="L8" s="6">
+      <c r="L9" s="6">
         <v>89</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A9">
+    <row r="10" spans="1:12">
+      <c r="A10">
         <v>2016</v>
       </c>
-      <c r="B9" s="6">
+      <c r="B10" s="6">
         <v>68</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C10" s="6">
         <v>109</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D10" s="6">
         <v>120</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E10" s="6">
         <v>98</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F10" s="6">
         <v>91</v>
       </c>
-      <c r="G9" s="6">
+      <c r="G10" s="6">
         <v>107</v>
       </c>
-      <c r="H9" s="6">
+      <c r="H10" s="6">
         <v>125</v>
       </c>
-      <c r="I9" s="6">
+      <c r="I10" s="6">
         <v>157</v>
       </c>
-      <c r="J9" s="6">
+      <c r="J10" s="6">
         <v>113</v>
       </c>
-      <c r="K9" s="6">
+      <c r="K10" s="6">
         <v>62</v>
       </c>
-      <c r="L9" s="6">
+      <c r="L10" s="6">
         <v>46</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A10">
+    <row r="11" spans="1:12">
+      <c r="A11">
         <v>2015</v>
       </c>
-      <c r="B10" s="6">
+      <c r="B11" s="6">
         <v>90</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C11" s="6">
         <v>136</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D11" s="6">
         <v>144</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E11" s="6">
         <v>123</v>
       </c>
-      <c r="F10" s="6">
+      <c r="F11" s="6">
         <v>57</v>
       </c>
-      <c r="G10" s="6">
+      <c r="G11" s="6">
         <v>95</v>
       </c>
-      <c r="H10" s="6">
+      <c r="H11" s="6">
         <v>106</v>
       </c>
-      <c r="I10" s="6">
+      <c r="I11" s="6">
         <v>156</v>
       </c>
-      <c r="J10" s="6">
+      <c r="J11" s="6">
         <v>141</v>
       </c>
-      <c r="K10" s="6">
+      <c r="K11" s="6">
         <v>73</v>
       </c>
-      <c r="L10" s="6">
+      <c r="L11" s="6">
         <v>47</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="L11" s="6"/>
+    <row r="12" spans="1:12">
+      <c r="L12" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -3313,9 +3461,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C84F5ED-A6BB-4026-BA10-F0FD0D737D80}">
   <dimension ref="A1:I7"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9">
       <c r="A1" s="10" t="s">
         <v>88</v>
       </c>
@@ -3344,7 +3492,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9">
       <c r="A2">
         <v>2015</v>
       </c>
@@ -3373,7 +3521,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9">
       <c r="A3">
         <v>2016</v>
       </c>
@@ -3402,7 +3550,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9">
       <c r="A4">
         <v>2017</v>
       </c>
@@ -3431,7 +3579,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9">
       <c r="A5">
         <v>2018</v>
       </c>
@@ -3460,7 +3608,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9">
       <c r="A6">
         <v>2019</v>
       </c>
@@ -3489,7 +3637,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9">
       <c r="A7">
         <v>2020</v>
       </c>
@@ -3526,10 +3674,10 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A633E54-D5CF-4061-865D-7F1B10E137A1}">
-  <dimension ref="A1:Q6"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:Q7"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:17">
       <c r="A1" s="10" t="s">
         <v>88</v>
       </c>
@@ -3582,268 +3730,321 @@
         <v>65</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A2" s="19">
+    <row r="2" spans="1:17">
+      <c r="A2" s="10">
+        <v>2023</v>
+      </c>
+      <c r="B2" s="4">
+        <v>35</v>
+      </c>
+      <c r="C2" s="5">
+        <v>205</v>
+      </c>
+      <c r="D2" s="5">
+        <v>289</v>
+      </c>
+      <c r="E2" s="5">
+        <v>110</v>
+      </c>
+      <c r="F2" s="5">
+        <v>48</v>
+      </c>
+      <c r="G2" s="5">
+        <v>39</v>
+      </c>
+      <c r="H2" s="5">
+        <v>45</v>
+      </c>
+      <c r="I2" s="5">
+        <v>45</v>
+      </c>
+      <c r="J2" s="5">
+        <v>25</v>
+      </c>
+      <c r="K2" s="5">
+        <v>32</v>
+      </c>
+      <c r="L2" s="5">
+        <v>35</v>
+      </c>
+      <c r="M2" s="5">
+        <v>23</v>
+      </c>
+      <c r="N2" s="5">
+        <v>19</v>
+      </c>
+      <c r="O2" s="5">
+        <v>10</v>
+      </c>
+      <c r="P2" s="5">
+        <v>13</v>
+      </c>
+      <c r="Q2" s="5">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17">
+      <c r="A3" s="19">
         <v>2022</v>
       </c>
-      <c r="B2">
+      <c r="B3">
         <v>28</v>
       </c>
-      <c r="C2">
+      <c r="C3">
         <v>103</v>
       </c>
-      <c r="D2">
+      <c r="D3">
         <v>86</v>
       </c>
-      <c r="E2">
+      <c r="E3">
         <v>44</v>
       </c>
-      <c r="F2">
+      <c r="F3">
         <v>18</v>
       </c>
-      <c r="G2">
+      <c r="G3">
         <v>17</v>
       </c>
-      <c r="H2">
+      <c r="H3">
         <v>30</v>
       </c>
-      <c r="I2">
+      <c r="I3">
         <v>23</v>
       </c>
-      <c r="J2">
+      <c r="J3">
         <v>22</v>
       </c>
-      <c r="K2">
+      <c r="K3">
         <v>25</v>
       </c>
-      <c r="L2">
+      <c r="L3">
         <v>21</v>
       </c>
-      <c r="M2">
+      <c r="M3">
         <v>12</v>
       </c>
-      <c r="N2">
+      <c r="N3">
         <v>6</v>
       </c>
-      <c r="O2">
+      <c r="O3">
         <v>14</v>
       </c>
-      <c r="P2">
+      <c r="P3">
         <v>6</v>
       </c>
-      <c r="Q2">
+      <c r="Q3">
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A3" s="19">
+    <row r="4" spans="1:17">
+      <c r="A4" s="19">
         <v>2021</v>
       </c>
-      <c r="B3">
+      <c r="B4">
         <v>30</v>
       </c>
-      <c r="C3">
+      <c r="C4">
         <v>175</v>
       </c>
-      <c r="D3">
+      <c r="D4">
         <v>113</v>
       </c>
-      <c r="E3">
+      <c r="E4">
         <v>56</v>
       </c>
-      <c r="F3">
+      <c r="F4">
         <v>31</v>
       </c>
-      <c r="G3">
+      <c r="G4">
         <v>40</v>
       </c>
-      <c r="H3">
+      <c r="H4">
         <v>47</v>
       </c>
-      <c r="I3">
+      <c r="I4">
         <v>45</v>
       </c>
-      <c r="J3">
+      <c r="J4">
         <v>34</v>
       </c>
-      <c r="K3">
+      <c r="K4">
         <v>40</v>
       </c>
-      <c r="L3">
+      <c r="L4">
         <v>20</v>
       </c>
-      <c r="M3">
+      <c r="M4">
         <v>18</v>
       </c>
-      <c r="N3">
+      <c r="N4">
         <v>17</v>
       </c>
-      <c r="O3">
+      <c r="O4">
         <v>12</v>
       </c>
-      <c r="P3">
+      <c r="P4">
         <v>5</v>
       </c>
-      <c r="Q3">
+      <c r="Q4">
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A4" s="19">
+    <row r="5" spans="1:17">
+      <c r="A5" s="19">
         <v>2020</v>
       </c>
-      <c r="B4">
+      <c r="B5">
         <v>162</v>
       </c>
-      <c r="C4">
+      <c r="C5">
         <v>189</v>
       </c>
-      <c r="D4">
+      <c r="D5">
         <v>803</v>
       </c>
-      <c r="E4">
+      <c r="E5">
         <v>606</v>
       </c>
-      <c r="F4">
+      <c r="F5">
         <v>113</v>
       </c>
-      <c r="G4">
+      <c r="G5">
         <v>69</v>
       </c>
-      <c r="H4">
+      <c r="H5">
         <v>82</v>
       </c>
-      <c r="I4">
+      <c r="I5">
         <v>114</v>
       </c>
-      <c r="J4">
+      <c r="J5">
         <v>119</v>
       </c>
-      <c r="K4">
+      <c r="K5">
         <v>154</v>
       </c>
-      <c r="L4">
+      <c r="L5">
         <v>132</v>
       </c>
-      <c r="M4">
+      <c r="M5">
         <v>72</v>
       </c>
-      <c r="N4">
+      <c r="N5">
         <v>51</v>
       </c>
-      <c r="O4">
+      <c r="O5">
         <v>39</v>
       </c>
-      <c r="P4">
+      <c r="P5">
         <v>36</v>
       </c>
-      <c r="Q4">
+      <c r="Q5">
         <v>78</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A5" s="19">
+    <row r="6" spans="1:17">
+      <c r="A6" s="19">
         <v>2019</v>
       </c>
-      <c r="B5">
+      <c r="B6">
         <v>878</v>
       </c>
-      <c r="C5">
+      <c r="C6">
         <v>815</v>
       </c>
-      <c r="D5">
+      <c r="D6">
         <v>5856</v>
       </c>
-      <c r="E5">
+      <c r="E6">
         <v>4489</v>
       </c>
-      <c r="F5">
+      <c r="F6">
         <v>664</v>
       </c>
-      <c r="G5">
+      <c r="G6">
         <v>282</v>
       </c>
-      <c r="H5">
+      <c r="H6">
         <v>366</v>
       </c>
-      <c r="I5">
+      <c r="I6">
         <v>373</v>
       </c>
-      <c r="J5">
+      <c r="J6">
         <v>526</v>
       </c>
-      <c r="K5">
+      <c r="K6">
         <v>695</v>
       </c>
-      <c r="L5">
+      <c r="L6">
         <v>572</v>
       </c>
-      <c r="M5">
+      <c r="M6">
         <v>317</v>
       </c>
-      <c r="N5">
+      <c r="N6">
         <v>225</v>
       </c>
-      <c r="O5">
+      <c r="O6">
         <v>201</v>
       </c>
-      <c r="P5">
+      <c r="P6">
         <v>205</v>
       </c>
-      <c r="Q5">
+      <c r="Q6">
         <v>381</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A6" s="19">
+    <row r="7" spans="1:17">
+      <c r="A7" s="19">
         <v>2018</v>
       </c>
-      <c r="B6">
+      <c r="B7">
         <v>619</v>
       </c>
-      <c r="C6">
+      <c r="C7">
         <v>614</v>
       </c>
-      <c r="D6">
+      <c r="D7">
         <v>4445</v>
       </c>
-      <c r="E6">
+      <c r="E7">
         <v>3036</v>
       </c>
-      <c r="F6">
+      <c r="F7">
         <v>413</v>
       </c>
-      <c r="G6">
+      <c r="G7">
         <v>216</v>
       </c>
-      <c r="H6">
+      <c r="H7">
         <v>214</v>
       </c>
-      <c r="I6">
+      <c r="I7">
         <v>283</v>
       </c>
-      <c r="J6">
+      <c r="J7">
         <v>441</v>
       </c>
-      <c r="K6">
+      <c r="K7">
         <v>503</v>
       </c>
-      <c r="L6">
+      <c r="L7">
         <v>390</v>
       </c>
-      <c r="M6">
+      <c r="M7">
         <v>215</v>
       </c>
-      <c r="N6">
+      <c r="N7">
         <v>176</v>
       </c>
-      <c r="O6">
+      <c r="O7">
         <v>137</v>
       </c>
-      <c r="P6">
+      <c r="P7">
         <v>145</v>
       </c>
-      <c r="Q6">
+      <c r="Q7">
         <v>268</v>
       </c>
     </row>
@@ -3855,10 +4056,10 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{336180FD-EF98-40EB-9484-811A5E7BC980}">
-  <dimension ref="A1:L10"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12">
       <c r="A1" s="10" t="s">
         <v>88</v>
       </c>
@@ -3896,345 +4097,394 @@
         <v>79</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A2" s="19">
+    <row r="2" spans="1:12">
+      <c r="A2" s="10">
+        <v>2024</v>
+      </c>
+      <c r="B2" s="20">
+        <f>2545*0.167</f>
+        <v>425.01500000000004</v>
+      </c>
+      <c r="C2" s="20">
+        <f>2545*0.047</f>
+        <v>119.61499999999999</v>
+      </c>
+      <c r="D2" s="20">
+        <f>2545*0.128</f>
+        <v>325.76</v>
+      </c>
+      <c r="E2" s="20">
+        <f>2545*0.077</f>
+        <v>195.965</v>
+      </c>
+      <c r="F2" s="20">
+        <f>2545*0.088</f>
+        <v>223.95999999999998</v>
+      </c>
+      <c r="G2" s="20">
+        <f>2545*0.119</f>
+        <v>302.85499999999996</v>
+      </c>
+      <c r="H2" s="20">
+        <f>2545*0.159</f>
+        <v>404.65500000000003</v>
+      </c>
+      <c r="I2" s="20">
+        <f>2545*0.102</f>
+        <v>259.58999999999997</v>
+      </c>
+      <c r="J2" s="20">
+        <f>2545*0.047</f>
+        <v>119.61499999999999</v>
+      </c>
+      <c r="K2" s="20">
+        <f>2545*0.033</f>
+        <v>83.984999999999999</v>
+      </c>
+      <c r="L2" s="20">
+        <f>2545*0.028</f>
+        <v>71.260000000000005</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" s="19">
         <v>2023</v>
       </c>
-      <c r="B2" s="20">
+      <c r="B3" s="20">
         <v>25.116</v>
       </c>
-      <c r="C2" s="20">
+      <c r="C3" s="20">
         <v>8.9700000000000006</v>
       </c>
-      <c r="D2" s="20">
+      <c r="D3" s="20">
         <v>18.077999999999999</v>
       </c>
-      <c r="E2" s="20">
+      <c r="E3" s="20">
         <v>12.005999999999998</v>
       </c>
-      <c r="F2" s="20">
+      <c r="F3" s="20">
         <v>11.040000000000001</v>
       </c>
-      <c r="G2" s="20">
+      <c r="G3" s="20">
         <v>8.9700000000000006</v>
       </c>
-      <c r="H2" s="20">
+      <c r="H3" s="20">
         <v>16.007999999999999</v>
       </c>
-      <c r="I2" s="20">
+      <c r="I3" s="20">
         <v>20.009999999999998</v>
       </c>
-      <c r="J2" s="20">
+      <c r="J3" s="20">
         <v>8.0039999999999996</v>
       </c>
-      <c r="K2" s="20">
+      <c r="K3" s="20">
         <v>4.968</v>
       </c>
-      <c r="L2" s="20">
+      <c r="L3" s="20">
         <v>4.0019999999999998</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A3" s="19">
+    <row r="4" spans="1:12">
+      <c r="A4" s="19">
         <v>2022</v>
       </c>
-      <c r="B3" s="20">
+      <c r="B4" s="20">
         <v>1.8359999999999999</v>
       </c>
-      <c r="C3" s="20">
+      <c r="C4" s="20">
         <v>0</v>
       </c>
-      <c r="D3" s="20">
+      <c r="D4" s="20">
         <v>0.91199999999999992</v>
       </c>
-      <c r="E3" s="20">
+      <c r="E4" s="20">
         <v>1.8359999999999999</v>
       </c>
-      <c r="F3" s="20">
+      <c r="F4" s="20">
         <v>0.91199999999999992</v>
       </c>
-      <c r="G3" s="20">
+      <c r="G4" s="20">
         <v>1.8359999999999999</v>
       </c>
-      <c r="H3" s="20">
+      <c r="H4" s="20">
         <v>0.91199999999999992</v>
       </c>
-      <c r="I3" s="20">
+      <c r="I4" s="20">
         <v>1.8359999999999999</v>
       </c>
-      <c r="J3" s="20">
+      <c r="J4" s="20">
         <v>0.91199999999999992</v>
       </c>
-      <c r="K3" s="20">
+      <c r="K4" s="20">
         <v>0</v>
       </c>
-      <c r="L3" s="20">
+      <c r="L4" s="20">
         <v>0.91199999999999992</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A4" s="19">
+    <row r="5" spans="1:12">
+      <c r="A5" s="19">
         <v>2021</v>
       </c>
-      <c r="B4" s="20">
+      <c r="B5" s="20">
         <v>1.9909999999999999</v>
       </c>
-      <c r="C4" s="20">
+      <c r="C5" s="20">
         <v>0.99</v>
       </c>
-      <c r="D4" s="20">
+      <c r="D5" s="20">
         <v>0</v>
       </c>
-      <c r="E4" s="20">
+      <c r="E5" s="20">
         <v>0.99</v>
       </c>
-      <c r="F4" s="20">
+      <c r="F5" s="20">
         <v>0.99</v>
       </c>
-      <c r="G4" s="20">
+      <c r="G5" s="20">
         <v>0</v>
       </c>
-      <c r="H4" s="20">
+      <c r="H5" s="20">
         <v>2.992</v>
       </c>
-      <c r="I4" s="20">
+      <c r="I5" s="20">
         <v>0.99</v>
       </c>
-      <c r="J4" s="20">
+      <c r="J5" s="20">
         <v>0</v>
       </c>
-      <c r="K4" s="20">
+      <c r="K5" s="20">
         <v>0.99</v>
       </c>
-      <c r="L4" s="20">
+      <c r="L5" s="20">
         <v>0.99</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A5" s="19">
+    <row r="6" spans="1:12">
+      <c r="A6" s="19">
         <v>2020</v>
       </c>
-      <c r="B5" s="20">
+      <c r="B6" s="20">
         <v>43.847000000000001</v>
       </c>
-      <c r="C5" s="20">
+      <c r="C6" s="20">
         <v>23.940999999999999</v>
       </c>
-      <c r="D5" s="20">
+      <c r="D6" s="20">
         <v>33.893999999999998</v>
       </c>
-      <c r="E5" s="20">
+      <c r="E6" s="20">
         <v>28.782999999999998</v>
       </c>
-      <c r="F5" s="20">
+      <c r="F6" s="20">
         <v>19.905999999999999</v>
       </c>
-      <c r="G5" s="20">
+      <c r="G6" s="20">
         <v>28.782999999999998</v>
       </c>
-      <c r="H5" s="20">
+      <c r="H6" s="20">
         <v>43.847000000000001</v>
       </c>
-      <c r="I5" s="20">
+      <c r="I6" s="20">
         <v>18.830000000000002</v>
       </c>
-      <c r="J5" s="20">
+      <c r="J6" s="20">
         <v>9.9529999999999994</v>
       </c>
-      <c r="K5" s="20">
+      <c r="K6" s="20">
         <v>7.8010000000000002</v>
       </c>
-      <c r="L5" s="20">
+      <c r="L6" s="20">
         <v>7.8010000000000002</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A6" s="19">
+    <row r="7" spans="1:12">
+      <c r="A7" s="19">
         <v>2019</v>
       </c>
-      <c r="B6" s="20">
+      <c r="B7" s="20">
         <v>105.57000000000001</v>
       </c>
-      <c r="C6" s="20">
+      <c r="C7" s="20">
         <v>38.318000000000005</v>
       </c>
-      <c r="D6" s="20">
+      <c r="D7" s="20">
         <v>84.456000000000003</v>
       </c>
-      <c r="E6" s="20">
+      <c r="E7" s="20">
         <v>68.816000000000003</v>
       </c>
-      <c r="F6" s="20">
+      <c r="F7" s="20">
         <v>107.91600000000001</v>
       </c>
-      <c r="G6" s="20">
+      <c r="G7" s="20">
         <v>81.328000000000003</v>
       </c>
-      <c r="H6" s="20">
+      <c r="H7" s="20">
         <v>135.286</v>
       </c>
-      <c r="I6" s="20">
+      <c r="I7" s="20">
         <v>79.763999999999996</v>
       </c>
-      <c r="J6" s="20">
+      <c r="J7" s="20">
         <v>34.408000000000001</v>
       </c>
-      <c r="K6" s="20">
+      <c r="K7" s="20">
         <v>32.844000000000001</v>
       </c>
-      <c r="L6" s="20">
+      <c r="L7" s="20">
         <v>8.6020000000000003</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A7" s="19">
+    <row r="8" spans="1:12">
+      <c r="A8" s="19">
         <v>2018</v>
       </c>
-      <c r="B7" s="20">
+      <c r="B8" s="20">
         <v>127.84699999999999</v>
       </c>
-      <c r="C7" s="20">
+      <c r="C8" s="20">
         <v>56.902999999999999</v>
       </c>
-      <c r="D7" s="20">
+      <c r="D8" s="20">
         <v>91.635999999999996</v>
       </c>
-      <c r="E7" s="20">
+      <c r="E8" s="20">
         <v>39.905999999999999</v>
       </c>
-      <c r="F7" s="20">
+      <c r="F8" s="20">
         <v>81.290000000000006</v>
       </c>
-      <c r="G7" s="20">
+      <c r="G8" s="20">
         <v>88.679999999999993</v>
       </c>
-      <c r="H7" s="20">
+      <c r="H8" s="20">
         <v>119.718</v>
       </c>
-      <c r="I7" s="20">
+      <c r="I8" s="20">
         <v>55.424999999999997</v>
       </c>
-      <c r="J7" s="20">
+      <c r="J8" s="20">
         <v>29.560000000000002</v>
       </c>
-      <c r="K7" s="20">
+      <c r="K8" s="20">
         <v>29.560000000000002</v>
       </c>
-      <c r="L7" s="20">
+      <c r="L8" s="20">
         <v>14.780000000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A8" s="19">
+    <row r="9" spans="1:12">
+      <c r="A9" s="19">
         <v>2017</v>
       </c>
-      <c r="B8" s="20">
+      <c r="B9" s="20">
         <v>132.82500000000002</v>
       </c>
-      <c r="C8" s="20">
+      <c r="C9" s="20">
         <v>46.690000000000005</v>
       </c>
-      <c r="D8" s="20">
+      <c r="D9" s="20">
         <v>109.48</v>
       </c>
-      <c r="E8" s="20">
+      <c r="E9" s="20">
         <v>57.959999999999994</v>
       </c>
-      <c r="F8" s="20">
+      <c r="F9" s="20">
         <v>82.914999999999992</v>
       </c>
-      <c r="G8" s="20">
+      <c r="G9" s="20">
         <v>90.965000000000003</v>
       </c>
-      <c r="H8" s="20">
+      <c r="H9" s="20">
         <v>124.77500000000001</v>
       </c>
-      <c r="I8" s="20">
+      <c r="I9" s="20">
         <v>64.400000000000006</v>
       </c>
-      <c r="J8" s="20">
+      <c r="J9" s="20">
         <v>38.64</v>
       </c>
-      <c r="K8" s="20">
+      <c r="K9" s="20">
         <v>38.64</v>
       </c>
-      <c r="L8" s="20">
+      <c r="L9" s="20">
         <v>14.489999999999998</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A9" s="19">
+    <row r="10" spans="1:12">
+      <c r="A10" s="19">
         <v>2016</v>
       </c>
-      <c r="B9" s="20">
+      <c r="B10" s="20">
         <v>126.973</v>
       </c>
-      <c r="C9" s="20">
+      <c r="C10" s="20">
         <v>46.851000000000006</v>
       </c>
-      <c r="D9" s="20">
+      <c r="D10" s="20">
         <v>72.652999999999992</v>
       </c>
-      <c r="E9" s="20">
+      <c r="E10" s="20">
         <v>61.789000000000001</v>
       </c>
-      <c r="F9" s="20">
+      <c r="F10" s="20">
         <v>84.875</v>
       </c>
-      <c r="G9" s="20">
+      <c r="G10" s="20">
         <v>79.442999999999998</v>
       </c>
-      <c r="H9" s="20">
+      <c r="H10" s="20">
         <v>91.665000000000006</v>
       </c>
-      <c r="I9" s="20">
+      <c r="I10" s="20">
         <v>41.418999999999997</v>
       </c>
-      <c r="J9" s="20">
+      <c r="J10" s="20">
         <v>33.950000000000003</v>
       </c>
-      <c r="K9" s="20">
+      <c r="K10" s="20">
         <v>29.875999999999998</v>
       </c>
-      <c r="L9" s="20">
+      <c r="L10" s="20">
         <v>6.79</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A10" s="19">
+    <row r="11" spans="1:12">
+      <c r="A11" s="19">
         <v>2015</v>
       </c>
-      <c r="B10" s="20">
+      <c r="B11" s="20">
         <v>127.23299999999999</v>
       </c>
-      <c r="C10" s="20">
+      <c r="C11" s="20">
         <v>37.386000000000003</v>
       </c>
-      <c r="D10" s="20">
+      <c r="D11" s="20">
         <v>42.812999999999995</v>
       </c>
-      <c r="E10" s="20">
+      <c r="E11" s="20">
         <v>61.505999999999993</v>
       </c>
-      <c r="F10" s="20">
+      <c r="F11" s="20">
         <v>76.581000000000003</v>
       </c>
-      <c r="G10" s="20">
+      <c r="G11" s="20">
         <v>74.772000000000006</v>
       </c>
-      <c r="H10" s="20">
+      <c r="H11" s="20">
         <v>79.596000000000004</v>
       </c>
-      <c r="I10" s="20">
+      <c r="I11" s="20">
         <v>37.386000000000003</v>
       </c>
-      <c r="J10" s="20">
+      <c r="J11" s="20">
         <v>36.783000000000001</v>
       </c>
-      <c r="K10" s="20">
+      <c r="K11" s="20">
         <v>18.693000000000001</v>
       </c>
-      <c r="L10" s="20">
+      <c r="L11" s="20">
         <v>6.633</v>
       </c>
     </row>

</xml_diff>